<commit_message>
feat: Game Feel 提升
</commit_message>
<xml_diff>
--- a/Tools/DataTablesTool/DataTables/Datas/#Sound.xlsx
+++ b/Tools/DataTablesTool/DataTables/Datas/#Sound.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="53">
   <si>
     <t>##var</t>
   </si>
@@ -169,13 +169,28 @@
     <t>Enemy Projectile Hit 2</t>
   </si>
   <si>
-    <t>Player Projectile</t>
-  </si>
-  <si>
     <t>Player Projectile Hit</t>
   </si>
   <si>
     <t>Player Dead</t>
+  </si>
+  <si>
+    <t>WeaponRifle</t>
+  </si>
+  <si>
+    <t>WeaponShotgun</t>
+  </si>
+  <si>
+    <t>WeaponRPG</t>
+  </si>
+  <si>
+    <t>WeaponEnergy</t>
+  </si>
+  <si>
+    <t>WeaponSniper</t>
+  </si>
+  <si>
+    <t>WeaponCrossbow</t>
   </si>
 </sst>
 </file>
@@ -644,148 +659,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1137,13 +1152,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="3" max="3" width="79.875" customWidth="1"/>
-    <col min="4" max="4" width="24.5" customWidth="1"/>
-    <col min="5" max="5" width="11.375" customWidth="1"/>
-    <col min="10" max="10" width="17.625" customWidth="1"/>
+    <col min="3" max="3" width="40.5" customWidth="1"/>
+    <col min="4" max="4" width="19.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -1336,7 +1349,7 @@
         <v>1</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1377,7 +1390,7 @@
         <v>1</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -1418,7 +1431,7 @@
         <v>0</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>0.65</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -1436,7 +1449,7 @@
         <v>0</v>
       </c>
       <c r="L7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M7">
         <v>100</v>
@@ -1459,7 +1472,7 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0.65</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -1477,7 +1490,7 @@
         <v>0</v>
       </c>
       <c r="L8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M8">
         <v>100</v>
@@ -1500,7 +1513,7 @@
         <v>0</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>0.65</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -1518,7 +1531,7 @@
         <v>0</v>
       </c>
       <c r="L9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M9">
         <v>100</v>
@@ -1541,7 +1554,7 @@
         <v>0</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0.65</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -1559,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="L10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10">
         <v>100</v>
@@ -1582,7 +1595,7 @@
         <v>0</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>0.65</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -1600,7 +1613,7 @@
         <v>0</v>
       </c>
       <c r="L11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11">
         <v>100</v>
@@ -1623,7 +1636,7 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0.65</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1641,7 +1654,7 @@
         <v>0</v>
       </c>
       <c r="L12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12">
         <v>100</v>
@@ -1664,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>0.65</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -1682,7 +1695,7 @@
         <v>0</v>
       </c>
       <c r="L13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13">
         <v>100</v>
@@ -1693,7 +1706,7 @@
     </row>
     <row r="14" spans="1:14">
       <c r="B14">
-        <v>2101</v>
+        <v>2102</v>
       </c>
       <c r="C14" t="s">
         <v>45</v>
@@ -1705,7 +1718,7 @@
         <v>0</v>
       </c>
       <c r="F14">
-        <v>1.5</v>
+        <v>0.65</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -1723,7 +1736,7 @@
         <v>0</v>
       </c>
       <c r="L14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M14">
         <v>100</v>
@@ -1734,7 +1747,7 @@
     </row>
     <row r="15" spans="1:14">
       <c r="B15">
-        <v>2102</v>
+        <v>2103</v>
       </c>
       <c r="C15" t="s">
         <v>46</v>
@@ -1764,7 +1777,7 @@
         <v>0</v>
       </c>
       <c r="L15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15">
         <v>100</v>
@@ -1775,7 +1788,7 @@
     </row>
     <row r="16" spans="1:14">
       <c r="B16">
-        <v>2103</v>
+        <v>2201</v>
       </c>
       <c r="C16" t="s">
         <v>47</v>
@@ -1805,12 +1818,217 @@
         <v>0</v>
       </c>
       <c r="L16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M16">
         <v>100</v>
       </c>
       <c r="N16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14">
+      <c r="B17">
+        <v>2202</v>
+      </c>
+      <c r="C17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" t="b">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0.8</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17">
+        <v>100</v>
+      </c>
+      <c r="N17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14">
+      <c r="B18">
+        <v>2203</v>
+      </c>
+      <c r="C18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>1</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>100</v>
+      </c>
+      <c r="N18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14">
+      <c r="B19">
+        <v>2204</v>
+      </c>
+      <c r="C19" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" t="s">
+        <v>38</v>
+      </c>
+      <c r="E19" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0.75</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>1</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>1</v>
+      </c>
+      <c r="M19">
+        <v>100</v>
+      </c>
+      <c r="N19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:14">
+      <c r="B20">
+        <v>2205</v>
+      </c>
+      <c r="C20" t="s">
+        <v>51</v>
+      </c>
+      <c r="D20" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20" t="b">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>1</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>1</v>
+      </c>
+      <c r="M20">
+        <v>100</v>
+      </c>
+      <c r="N20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="2:14">
+      <c r="B21">
+        <v>2206</v>
+      </c>
+      <c r="C21" t="s">
+        <v>52</v>
+      </c>
+      <c r="D21" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0.9</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>1</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21">
+        <v>100</v>
+      </c>
+      <c r="N21">
         <v>1</v>
       </c>
     </row>

</xml_diff>